<commit_message>
Add INA219 and ESP8266 drivers with Open/Ioctl/Read/Write API, update FreeRTOS tasks, fix TIM3 servo control
</commit_message>
<xml_diff>
--- a/Pm.xlsx
+++ b/Pm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/makbuleozler/Desktop/Embedded_Projects/ELE529E_SolarTracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED9CE76-77EC-8C42-A471-776CCBE42C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{896301FE-1F14-7B4A-886E-72D559245FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{CB9406A4-677C-0942-BB42-658C862FF8FD}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="v1" sheetId="1" r:id="rId1"/>
     <sheet name="v2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -678,51 +678,54 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -730,9 +733,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1669,472 +1669,472 @@
       </c>
     </row>
     <row r="5" spans="4:8" ht="52">
-      <c r="D5" s="7">
+      <c r="D5" s="12">
         <v>1</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="21" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="4:8" ht="25">
-      <c r="D6" s="12"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="16"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="4:8" ht="52">
-      <c r="D7" s="12"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="17" t="s">
+      <c r="D7" s="13"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="16"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="22"/>
     </row>
     <row r="8" spans="4:8" ht="25">
-      <c r="D8" s="12"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="16"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="22"/>
     </row>
     <row r="9" spans="4:8" ht="26">
-      <c r="D9" s="12"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="17" t="s">
+      <c r="D9" s="13"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="16"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="22"/>
     </row>
     <row r="10" spans="4:8" ht="25">
-      <c r="D10" s="12"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="16"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="22"/>
     </row>
     <row r="11" spans="4:8" ht="52">
-      <c r="D11" s="12"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="17" t="s">
+      <c r="D11" s="13"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="15"/>
-      <c r="H11" s="16"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="22"/>
     </row>
     <row r="12" spans="4:8" ht="25">
-      <c r="D12" s="12"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="16"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="22"/>
     </row>
     <row r="13" spans="4:8" ht="52">
-      <c r="D13" s="18"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="20" t="s">
+      <c r="D13" s="14"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="G13" s="21"/>
-      <c r="H13" s="22"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="23"/>
     </row>
     <row r="14" spans="4:8" ht="52">
-      <c r="D14" s="7">
+      <c r="D14" s="12">
         <v>2</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="21" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="15" spans="4:8" ht="25">
-      <c r="D15" s="12"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="16"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="22"/>
     </row>
     <row r="16" spans="4:8" ht="52">
-      <c r="D16" s="12"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="17" t="s">
+      <c r="D16" s="13"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="16"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="22"/>
     </row>
     <row r="17" spans="4:8" ht="25">
-      <c r="D17" s="12"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="16"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="22"/>
     </row>
     <row r="18" spans="4:8" ht="52">
-      <c r="D18" s="12"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="17" t="s">
+      <c r="D18" s="13"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="G18" s="15"/>
-      <c r="H18" s="16"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="22"/>
     </row>
     <row r="19" spans="4:8" ht="25">
-      <c r="D19" s="12"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="16"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="22"/>
     </row>
     <row r="20" spans="4:8" ht="52">
-      <c r="D20" s="18"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="20" t="s">
+      <c r="D20" s="14"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="G20" s="21"/>
-      <c r="H20" s="22"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="23"/>
     </row>
     <row r="21" spans="4:8" ht="26">
-      <c r="D21" s="7">
+      <c r="D21" s="12">
         <v>3</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="G21" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="H21" s="21" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="22" spans="4:8" ht="25">
-      <c r="D22" s="12"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="16"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="22"/>
     </row>
     <row r="23" spans="4:8" ht="26">
-      <c r="D23" s="12"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="17" t="s">
+      <c r="D23" s="13"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="G23" s="15"/>
-      <c r="H23" s="16"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="22"/>
     </row>
     <row r="24" spans="4:8" ht="25">
-      <c r="D24" s="12"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="16"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="22"/>
     </row>
     <row r="25" spans="4:8" ht="52">
-      <c r="D25" s="12"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="17" t="s">
+      <c r="D25" s="13"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="G25" s="15"/>
-      <c r="H25" s="16"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="22"/>
     </row>
     <row r="26" spans="4:8" ht="25">
-      <c r="D26" s="12"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="16"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="22"/>
     </row>
     <row r="27" spans="4:8" ht="52">
-      <c r="D27" s="18"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="20" t="s">
+      <c r="D27" s="14"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="G27" s="21"/>
-      <c r="H27" s="22"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="23"/>
     </row>
     <row r="28" spans="4:8" ht="52">
-      <c r="D28" s="7">
+      <c r="D28" s="12">
         <v>4</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="F28" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="G28" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="H28" s="11" t="s">
+      <c r="H28" s="21" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="29" spans="4:8" ht="25">
-      <c r="D29" s="12"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="16"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="22"/>
     </row>
     <row r="30" spans="4:8" ht="52">
-      <c r="D30" s="12"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="17" t="s">
+      <c r="D30" s="13"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="G30" s="15"/>
-      <c r="H30" s="16"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="22"/>
     </row>
     <row r="31" spans="4:8" ht="25">
-      <c r="D31" s="12"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="16"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="22"/>
     </row>
     <row r="32" spans="4:8" ht="52">
-      <c r="D32" s="18"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="20" t="s">
+      <c r="D32" s="14"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="G32" s="21"/>
-      <c r="H32" s="22"/>
+      <c r="G32" s="20"/>
+      <c r="H32" s="23"/>
     </row>
     <row r="33" spans="4:8" ht="26">
-      <c r="D33" s="7">
+      <c r="D33" s="12">
         <v>5</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="G33" s="10" t="s">
+      <c r="G33" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="H33" s="11" t="s">
+      <c r="H33" s="21" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="34" spans="4:8" ht="25">
-      <c r="D34" s="12"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="16"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="22"/>
     </row>
     <row r="35" spans="4:8" ht="52">
-      <c r="D35" s="12"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="17" t="s">
+      <c r="D35" s="13"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="G35" s="15"/>
-      <c r="H35" s="16"/>
+      <c r="G35" s="19"/>
+      <c r="H35" s="22"/>
     </row>
     <row r="36" spans="4:8" ht="25">
-      <c r="D36" s="12"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="15"/>
-      <c r="H36" s="16"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="19"/>
+      <c r="H36" s="22"/>
     </row>
     <row r="37" spans="4:8" ht="52">
-      <c r="D37" s="12"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="17" t="s">
+      <c r="D37" s="13"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G37" s="15"/>
-      <c r="H37" s="16"/>
+      <c r="G37" s="19"/>
+      <c r="H37" s="22"/>
     </row>
     <row r="38" spans="4:8" ht="25">
-      <c r="D38" s="12"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="15"/>
-      <c r="H38" s="16"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="22"/>
     </row>
     <row r="39" spans="4:8" ht="52">
-      <c r="D39" s="18"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="20" t="s">
+      <c r="D39" s="14"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="G39" s="21"/>
-      <c r="H39" s="22"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="23"/>
     </row>
     <row r="40" spans="4:8" ht="52">
-      <c r="D40" s="7">
+      <c r="D40" s="12">
         <v>6</v>
       </c>
-      <c r="E40" s="8" t="s">
+      <c r="E40" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="F40" s="9" t="s">
+      <c r="F40" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="G40" s="10" t="s">
+      <c r="G40" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="H40" s="11" t="s">
+      <c r="H40" s="21" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="41" spans="4:8" ht="25">
-      <c r="D41" s="12"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="16"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="16"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="22"/>
     </row>
     <row r="42" spans="4:8" ht="26">
-      <c r="D42" s="12"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="17" t="s">
+      <c r="D42" s="13"/>
+      <c r="E42" s="16"/>
+      <c r="F42" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="G42" s="15"/>
-      <c r="H42" s="16"/>
+      <c r="G42" s="19"/>
+      <c r="H42" s="22"/>
     </row>
     <row r="43" spans="4:8" ht="25">
-      <c r="D43" s="12"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="16"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="19"/>
+      <c r="H43" s="22"/>
     </row>
     <row r="44" spans="4:8" ht="52">
-      <c r="D44" s="18"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="20" t="s">
+      <c r="D44" s="14"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="G44" s="21"/>
-      <c r="H44" s="22"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="23"/>
     </row>
     <row r="45" spans="4:8" ht="52">
-      <c r="D45" s="7">
+      <c r="D45" s="12">
         <v>7</v>
       </c>
-      <c r="E45" s="8" t="s">
+      <c r="E45" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F45" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="G45" s="10" t="s">
+      <c r="G45" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="H45" s="11" t="s">
+      <c r="H45" s="21" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="46" spans="4:8" ht="25">
-      <c r="D46" s="12"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="16"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="19"/>
+      <c r="H46" s="22"/>
     </row>
     <row r="47" spans="4:8" ht="52">
-      <c r="D47" s="12"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="17" t="s">
+      <c r="D47" s="13"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="G47" s="15"/>
-      <c r="H47" s="16"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="22"/>
     </row>
     <row r="48" spans="4:8" ht="25">
-      <c r="D48" s="12"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="15"/>
-      <c r="H48" s="16"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="16"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="19"/>
+      <c r="H48" s="22"/>
     </row>
     <row r="49" spans="4:8" ht="52">
-      <c r="D49" s="18"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="20" t="s">
+      <c r="D49" s="14"/>
+      <c r="E49" s="17"/>
+      <c r="F49" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="G49" s="21"/>
-      <c r="H49" s="22"/>
+      <c r="G49" s="20"/>
+      <c r="H49" s="23"/>
     </row>
     <row r="50" spans="4:8" ht="26">
-      <c r="D50" s="12">
+      <c r="D50" s="13">
         <v>8</v>
       </c>
-      <c r="E50" s="13" t="s">
+      <c r="E50" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="F50" s="17" t="s">
+      <c r="F50" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="G50" s="15" t="s">
+      <c r="G50" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="H50" s="16" t="s">
+      <c r="H50" s="22" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="51" spans="4:8" ht="25">
-      <c r="D51" s="12"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="15"/>
-      <c r="H51" s="16"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="16"/>
+      <c r="F51" s="8"/>
+      <c r="G51" s="19"/>
+      <c r="H51" s="22"/>
     </row>
     <row r="52" spans="4:8" ht="52">
-      <c r="D52" s="12"/>
-      <c r="E52" s="13"/>
-      <c r="F52" s="17" t="s">
+      <c r="D52" s="13"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="G52" s="15"/>
-      <c r="H52" s="16"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="22"/>
     </row>
     <row r="53" spans="4:8" ht="25">
-      <c r="D53" s="12"/>
-      <c r="E53" s="13"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="15"/>
-      <c r="H53" s="16"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="16"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="19"/>
+      <c r="H53" s="22"/>
     </row>
     <row r="54" spans="4:8" ht="53" thickBot="1">
-      <c r="D54" s="23"/>
-      <c r="E54" s="24"/>
-      <c r="F54" s="25" t="s">
+      <c r="D54" s="24"/>
+      <c r="E54" s="25"/>
+      <c r="F54" s="11" t="s">
         <v>105</v>
       </c>
       <c r="G54" s="26"/>
@@ -2142,6 +2142,30 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="D45:D49"/>
+    <mergeCell ref="E45:E49"/>
+    <mergeCell ref="G45:G49"/>
+    <mergeCell ref="H45:H49"/>
+    <mergeCell ref="D50:D54"/>
+    <mergeCell ref="E50:E54"/>
+    <mergeCell ref="G50:G54"/>
+    <mergeCell ref="H50:H54"/>
+    <mergeCell ref="D33:D39"/>
+    <mergeCell ref="E33:E39"/>
+    <mergeCell ref="G33:G39"/>
+    <mergeCell ref="H33:H39"/>
+    <mergeCell ref="D40:D44"/>
+    <mergeCell ref="E40:E44"/>
+    <mergeCell ref="G40:G44"/>
+    <mergeCell ref="H40:H44"/>
+    <mergeCell ref="D21:D27"/>
+    <mergeCell ref="E21:E27"/>
+    <mergeCell ref="G21:G27"/>
+    <mergeCell ref="H21:H27"/>
+    <mergeCell ref="D28:D32"/>
+    <mergeCell ref="E28:E32"/>
+    <mergeCell ref="G28:G32"/>
+    <mergeCell ref="H28:H32"/>
     <mergeCell ref="D5:D13"/>
     <mergeCell ref="E5:E13"/>
     <mergeCell ref="G5:G13"/>
@@ -2150,30 +2174,6 @@
     <mergeCell ref="E14:E20"/>
     <mergeCell ref="G14:G20"/>
     <mergeCell ref="H14:H20"/>
-    <mergeCell ref="D21:D27"/>
-    <mergeCell ref="E21:E27"/>
-    <mergeCell ref="G21:G27"/>
-    <mergeCell ref="H21:H27"/>
-    <mergeCell ref="D28:D32"/>
-    <mergeCell ref="E28:E32"/>
-    <mergeCell ref="G28:G32"/>
-    <mergeCell ref="H28:H32"/>
-    <mergeCell ref="D33:D39"/>
-    <mergeCell ref="E33:E39"/>
-    <mergeCell ref="G33:G39"/>
-    <mergeCell ref="H33:H39"/>
-    <mergeCell ref="D40:D44"/>
-    <mergeCell ref="E40:E44"/>
-    <mergeCell ref="G40:G44"/>
-    <mergeCell ref="H40:H44"/>
-    <mergeCell ref="D45:D49"/>
-    <mergeCell ref="E45:E49"/>
-    <mergeCell ref="G45:G49"/>
-    <mergeCell ref="H45:H49"/>
-    <mergeCell ref="D50:D54"/>
-    <mergeCell ref="E50:E54"/>
-    <mergeCell ref="G50:G54"/>
-    <mergeCell ref="H50:H54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="39" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>